<commit_message>
POWELL BIOFAC MARCH 25
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61334A7B-CC61-4144-8899-50A4605B449F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB846E59-6434-4194-8F04-986B77735589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13875" yWindow="0" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="720" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="128">
   <si>
     <t>Date</t>
   </si>
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G346"/>
+  <dimension ref="A1:G347"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8258,7 +8258,7 @@
         <v>2212.31</v>
       </c>
       <c r="D341">
-        <f>100*(B341-C341)/C341</f>
+        <f t="shared" ref="D341:D347" si="16">100*(B341-C341)/C341</f>
         <v>-5.0096505462621628E-2</v>
       </c>
       <c r="E341">
@@ -8279,7 +8279,7 @@
         <v>2212.31</v>
       </c>
       <c r="D342">
-        <f>100*(B342-C342)/C342</f>
+        <f t="shared" si="16"/>
         <v>0.45164782512396029</v>
       </c>
       <c r="E342">
@@ -8300,7 +8300,7 @@
         <v>2212.31</v>
       </c>
       <c r="D343">
-        <f>100*(B343-C343)/C343</f>
+        <f t="shared" si="16"/>
         <v>0.88534699025001196</v>
       </c>
       <c r="E343">
@@ -8321,7 +8321,7 @@
         <v>2212.31</v>
       </c>
       <c r="D344">
-        <f>100*(B344-C344)/C344</f>
+        <f t="shared" si="16"/>
         <v>0.38471507157676671</v>
       </c>
       <c r="E344">
@@ -8342,7 +8342,7 @@
         <v>2212.31</v>
       </c>
       <c r="D345">
-        <f>100*(B345-C345)/C345</f>
+        <f t="shared" si="16"/>
         <v>-5.1107665743038141E-2</v>
       </c>
       <c r="E345">
@@ -8363,7 +8363,7 @@
         <v>2212.31</v>
       </c>
       <c r="D346">
-        <f>100*(B346-C346)/C346</f>
+        <f t="shared" si="16"/>
         <v>-0.50397322255922039</v>
       </c>
       <c r="E346">
@@ -8371,6 +8371,27 @@
       </c>
       <c r="F346" t="s">
         <v>127</v>
+      </c>
+    </row>
+    <row r="347" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A347" s="1">
+        <v>46280</v>
+      </c>
+      <c r="B347" s="2">
+        <v>2209.8926799999999</v>
+      </c>
+      <c r="C347">
+        <v>2212.31</v>
+      </c>
+      <c r="D347">
+        <f t="shared" si="16"/>
+        <v>-0.10926678449222839</v>
+      </c>
+      <c r="E347">
+        <v>217</v>
+      </c>
+      <c r="F347" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
POWELL MARCH 25 2100
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB846E59-6434-4194-8F04-986B77735589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4393DDEF-1B2E-46E8-89AC-869AB097CF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="720" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13680" yWindow="510" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="128">
   <si>
     <t>Date</t>
   </si>
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G347"/>
+  <dimension ref="A1:G348"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8258,7 +8258,7 @@
         <v>2212.31</v>
       </c>
       <c r="D341">
-        <f t="shared" ref="D341:D347" si="16">100*(B341-C341)/C341</f>
+        <f t="shared" ref="D341:D348" si="16">100*(B341-C341)/C341</f>
         <v>-5.0096505462621628E-2</v>
       </c>
       <c r="E341">
@@ -8391,6 +8391,27 @@
         <v>217</v>
       </c>
       <c r="F347" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A348" s="1">
+        <v>46281</v>
+      </c>
+      <c r="B348" s="2">
+        <v>2209.0641000000001</v>
+      </c>
+      <c r="C348">
+        <v>2212.31</v>
+      </c>
+      <c r="D348">
+        <f t="shared" si="16"/>
+        <v>-0.14671994431159704</v>
+      </c>
+      <c r="E348">
+        <v>217</v>
+      </c>
+      <c r="F348" t="s">
         <v>125</v>
       </c>
     </row>

</xml_diff>

<commit_message>
POWELL APRIL 1 2026 BIOFAC
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4393DDEF-1B2E-46E8-89AC-869AB097CF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9840798C-3758-41C6-A1D3-2C44CCDD34EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13680" yWindow="510" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13875" yWindow="0" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="129">
   <si>
     <t>Date</t>
   </si>
@@ -417,6 +417,9 @@
   </si>
   <si>
     <t>same CRM opened 08/27/2026, New pH probe</t>
+  </si>
+  <si>
+    <t>new CRM opened 9/18/2026</t>
   </si>
 </sst>
 </file>
@@ -1282,7 +1285,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G348"/>
+  <dimension ref="A1:G349"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8258,7 +8261,7 @@
         <v>2212.31</v>
       </c>
       <c r="D341">
-        <f t="shared" ref="D341:D348" si="16">100*(B341-C341)/C341</f>
+        <f t="shared" ref="D341:D349" si="16">100*(B341-C341)/C341</f>
         <v>-5.0096505462621628E-2</v>
       </c>
       <c r="E341">
@@ -8413,6 +8416,27 @@
       </c>
       <c r="F348" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A349" s="1">
+        <v>46283</v>
+      </c>
+      <c r="B349" s="2">
+        <v>2207.9616700000001</v>
+      </c>
+      <c r="C349">
+        <v>2212.31</v>
+      </c>
+      <c r="D349">
+        <f t="shared" si="16"/>
+        <v>-0.19655156827026074</v>
+      </c>
+      <c r="E349">
+        <v>217</v>
+      </c>
+      <c r="F349" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating 9/18 data calcs with correct ph cal
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9840798C-3758-41C6-A1D3-2C44CCDD34EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE2B8BC-6CA8-499C-A3E4-CA1E8C79A17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13875" yWindow="0" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8423,14 +8423,14 @@
         <v>46283</v>
       </c>
       <c r="B349" s="2">
-        <v>2207.9616700000001</v>
+        <v>2209.1144800000002</v>
       </c>
       <c r="C349">
         <v>2212.31</v>
       </c>
       <c r="D349">
         <f t="shared" si="16"/>
-        <v>-0.19655156827026074</v>
+        <v>-0.1444426866035845</v>
       </c>
       <c r="E349">
         <v>217</v>

</xml_diff>

<commit_message>
POWELL APRIL 1 2100 BIOFAC
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE2B8BC-6CA8-499C-A3E4-CA1E8C79A17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71EB93F7-2DC0-408A-B825-E404307912BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13875" yWindow="0" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="130">
   <si>
     <t>Date</t>
   </si>
@@ -420,6 +420,9 @@
   </si>
   <si>
     <t>new CRM opened 9/18/2026</t>
+  </si>
+  <si>
+    <t>same CRM opened 9/18/2026</t>
   </si>
 </sst>
 </file>
@@ -1285,7 +1288,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G349"/>
+  <dimension ref="A1:G350"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8261,7 +8264,7 @@
         <v>2212.31</v>
       </c>
       <c r="D341">
-        <f t="shared" ref="D341:D349" si="16">100*(B341-C341)/C341</f>
+        <f t="shared" ref="D341:D350" si="16">100*(B341-C341)/C341</f>
         <v>-5.0096505462621628E-2</v>
       </c>
       <c r="E341">
@@ -8437,6 +8440,27 @@
       </c>
       <c r="F349" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="350" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A350" s="1">
+        <v>46286</v>
+      </c>
+      <c r="B350" s="2">
+        <v>2213.4127100000001</v>
+      </c>
+      <c r="C350">
+        <v>2212.31</v>
+      </c>
+      <c r="D350">
+        <f t="shared" si="16"/>
+        <v>4.9844280412786435E-2</v>
+      </c>
+      <c r="E350">
+        <v>217</v>
+      </c>
+      <c r="F350" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
POWELL BIOFAC APRIL 27 1200 AND 2100
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71EB93F7-2DC0-408A-B825-E404307912BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE790A2A-A0E8-4AB9-8FE8-8D946BA43E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13875" yWindow="0" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="720" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="130">
   <si>
     <t>Date</t>
   </si>
@@ -1288,7 +1288,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G350"/>
+  <dimension ref="A1:G351"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8264,7 +8264,7 @@
         <v>2212.31</v>
       </c>
       <c r="D341">
-        <f t="shared" ref="D341:D350" si="16">100*(B341-C341)/C341</f>
+        <f t="shared" ref="D341:D351" si="16">100*(B341-C341)/C341</f>
         <v>-5.0096505462621628E-2</v>
       </c>
       <c r="E341">
@@ -8460,6 +8460,27 @@
         <v>217</v>
       </c>
       <c r="F350" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A351" s="1">
+        <v>46287</v>
+      </c>
+      <c r="B351" s="2">
+        <v>2217.68084</v>
+      </c>
+      <c r="C351">
+        <v>2212.31</v>
+      </c>
+      <c r="D351">
+        <f t="shared" si="16"/>
+        <v>0.24277067861195059</v>
+      </c>
+      <c r="E351">
+        <v>217</v>
+      </c>
+      <c r="F351" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
powell biofac april 13th data 1200 and 2100
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE790A2A-A0E8-4AB9-8FE8-8D946BA43E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7048727F-B9B9-4909-9FF6-717C1F0B0088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="720" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13965" yWindow="0" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="131">
   <si>
     <t>Date</t>
   </si>
@@ -423,6 +423,9 @@
   </si>
   <si>
     <t>same CRM opened 9/18/2026</t>
+  </si>
+  <si>
+    <t>same CRM opened 9/18/2026, MP ran at end of 62 samples</t>
   </si>
 </sst>
 </file>
@@ -1288,7 +1291,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G351"/>
+  <dimension ref="A1:G353"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8264,7 +8267,7 @@
         <v>2212.31</v>
       </c>
       <c r="D341">
-        <f t="shared" ref="D341:D351" si="16">100*(B341-C341)/C341</f>
+        <f t="shared" ref="D341:D353" si="16">100*(B341-C341)/C341</f>
         <v>-5.0096505462621628E-2</v>
       </c>
       <c r="E341">
@@ -8482,6 +8485,48 @@
       </c>
       <c r="F351" t="s">
         <v>129</v>
+      </c>
+    </row>
+    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A352" s="1">
+        <v>46314</v>
+      </c>
+      <c r="B352" s="2">
+        <v>2209.7436200000002</v>
+      </c>
+      <c r="C352">
+        <v>2212.31</v>
+      </c>
+      <c r="D352">
+        <f t="shared" si="16"/>
+        <v>-0.11600453824282102</v>
+      </c>
+      <c r="E352">
+        <v>217</v>
+      </c>
+      <c r="F352" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="353" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A353" s="1">
+        <v>46314</v>
+      </c>
+      <c r="B353" s="2">
+        <v>2213.4907400000002</v>
+      </c>
+      <c r="C353">
+        <v>2212.31</v>
+      </c>
+      <c r="D353">
+        <f t="shared" si="16"/>
+        <v>5.3371362964514092E-2</v>
+      </c>
+      <c r="E353">
+        <v>217</v>
+      </c>
+      <c r="F353" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DMB update Metrohm titrant concentration and density equation. TA testing files and first round of DMB samples
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2C5D31-A81C-4CA6-B3C6-AFB3244975D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A253647-4D84-47AF-B357-9DFC74749718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13605" yWindow="690" windowWidth="14775" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="720" windowWidth="17145" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="132">
   <si>
     <t>Date</t>
   </si>
@@ -425,7 +425,10 @@
     <t>same CRM opened 9/18/2026, MP ran at end of 62 samples</t>
   </si>
   <si>
-    <t>same CRM opened 9/18/2026 - testing Metrohm acid</t>
+    <t>new CRM opened 10/28/2026. using Metrohm titrant w/ concentration=0.101125</t>
+  </si>
+  <si>
+    <t>same CRM opened 10/28/2026</t>
   </si>
 </sst>
 </file>
@@ -8267,7 +8270,7 @@
         <v>2212.31</v>
       </c>
       <c r="D341">
-        <f t="shared" ref="D341:D356" si="16">100*(B341-C341)/C341</f>
+        <f t="shared" ref="D341:D355" si="16">100*(B341-C341)/C341</f>
         <v>-5.0096505462621628E-2</v>
       </c>
       <c r="E341">
@@ -8552,20 +8555,20 @@
     </row>
     <row r="355" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A355" s="1">
-        <v>46321</v>
-      </c>
-      <c r="B355" s="2">
-        <v>2218.9580000000001</v>
+        <v>46323</v>
+      </c>
+      <c r="B355">
+        <v>2208.2145607079701</v>
       </c>
       <c r="C355">
-        <v>2212.31</v>
+        <v>2210.1999999999998</v>
       </c>
       <c r="D355">
         <f t="shared" si="16"/>
-        <v>0.30050038195371076</v>
+        <v>-8.9830752512428558E-2</v>
       </c>
       <c r="E355">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="F355" t="s">
         <v>130</v>
@@ -8573,23 +8576,23 @@
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A356" s="1">
-        <v>46321</v>
-      </c>
-      <c r="B356" s="2">
-        <v>2247.77</v>
+        <v>46324</v>
+      </c>
+      <c r="B356">
+        <v>2208.9469234640601</v>
       </c>
       <c r="C356">
-        <v>2212.31</v>
+        <v>2210.1999999999998</v>
       </c>
       <c r="D356">
-        <f t="shared" si="16"/>
-        <v>1.6028495102404292</v>
+        <f t="shared" ref="D356" si="17">100*(B356-C356)/C356</f>
+        <v>-5.6695164959719782E-2</v>
       </c>
       <c r="E356">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="F356" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DMB 10/30/2026 hawaii BEF
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A253647-4D84-47AF-B357-9DFC74749718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC1504B-2E59-4A36-981D-8B2811E023A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="720" windowWidth="17145" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="720" windowWidth="17145" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="132">
   <si>
     <t>Date</t>
   </si>
@@ -1294,7 +1294,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G356"/>
+  <dimension ref="A1:G357"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8595,6 +8595,27 @@
         <v>131</v>
       </c>
     </row>
+    <row r="357" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A357" s="1">
+        <v>46325</v>
+      </c>
+      <c r="B357">
+        <v>2227.0935546189598</v>
+      </c>
+      <c r="C357">
+        <v>2210.1999999999998</v>
+      </c>
+      <c r="D357">
+        <f t="shared" ref="D357" si="18">100*(B357-C357)/C357</f>
+        <v>0.7643450646529738</v>
+      </c>
+      <c r="E357">
+        <v>227</v>
+      </c>
+      <c r="F357" t="s">
+        <v>131</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>